<commit_message>
Updated SCoC and PLANAbPiaSY files
</commit_message>
<xml_diff>
--- a/InputData/land/PLANAbPiaSY/Potential Land Area Newly Affected by Pol in a Single Yr.xlsx
+++ b/InputData/land/PLANAbPiaSY/Potential Land Area Newly Affected by Pol in a Single Yr.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minhe\Dropbox\01. NEXT Group\00. NEXT Group\20. 프로젝트 관리\2025 에너지 수요전망 모형 구축\EPS 모형\eps-southkorea-3.3.1\InputData\land\PLANAbPiaSY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\administer\Dropbox\kjh\2025\02. EPS\EI\251119_메일회신\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C0E710C-42E5-4D8F-9EEE-185E03618C1E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56422AF8-C8D7-4E8D-A7B2-D7EC6EC67127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15405" yWindow="105" windowWidth="22635" windowHeight="20520" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="777" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -19,17 +19,31 @@
     <sheet name="Avoided Def" sheetId="7" r:id="rId4"/>
     <sheet name="Impr Forest Mgmt" sheetId="9" r:id="rId5"/>
     <sheet name="Forest Restoration" sheetId="10" r:id="rId6"/>
-    <sheet name="PLANAbPiaSY" sheetId="3" r:id="rId7"/>
+    <sheet name="Peatland Restoration" sheetId="13" r:id="rId7"/>
+    <sheet name="PLANAbPiaSY" sheetId="3" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="acres_per_million_hectares">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="129">
   <si>
     <t>PLANAbPiaSY Potential Land Area Newly Affected by Policy in a Single Year</t>
   </si>
@@ -397,18 +411,173 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
+    <t>E 나라지표</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Page 20, 2020 소유별 산림현황 및 산림비율</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Page 192, 산림복원 현황</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
     <t>https://www.index.go.kr/unity/potal/main/EachDtlPageDetail.do?idx_cd=1304</t>
-  </si>
-  <si>
-    <t>E 나라지표</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>Page 20, 2020 소유별 산림현황 및 산림비율</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>Page 192, 산림복원 현황</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Impr Wetland Mgmt</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>km2</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Measure</t>
+  </si>
+  <si>
+    <t>Acres Covered</t>
+  </si>
+  <si>
+    <t>Restoring Wetlands</t>
+  </si>
+  <si>
+    <t>Restoring Riparian Forest Buffers</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (acres/year)</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>(31페이지) - 2. 습지의 실표적 보전관리/ 연안습지 복원면적</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>제4차 습지보전기본계획(2023~2027)</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.mcee.go.kr/home/web/policy_data/read.do?menuId=10261&amp;seq=7993</t>
+  </si>
+  <si>
+    <t>note</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>- 연안습지 복원 '25년까지 4.5㎢(갯벌기본계획 목표 연계), '27년 7㎢ 복원 목표 및 갯벌 식생 복원 사업 확대 시행('27년 60㎢)</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. 제4차 습지보전기본계획(2023~2027)(31페이지) - 2. 습지의 실효적 보전관리/ 연안습지 복원면적 기준 계획</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>acres</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2050년까지 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>블루카본 부문에서 1.362 MtCO₂eq 흡수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>를 목표로 하면서,</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">이를 위해 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>폐염전·폐어장 등을 활용해 2050년까지 갯벌 30 km²를 복원</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>하고, 잘피 군락도 확대하겠다고 명시함</t>
+    </r>
+  </si>
+  <si>
+    <t>2027년</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>2050년</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Total Divided Over Years</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>2023~2027</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>2028~2050</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>2. IMO 제출용 [Toward Green Shipping by 2050] 에서 2050년 목표 언급</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>This study utilized two official sources to set the mid-to-long-term wetland restoration potential for South Korea.</t>
+  </si>
+  <si>
+    <t>Impr Peatland Restoration</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Korea has expanded this policy (peatland restoration) to encompass overall wetland restoration efforts.</t>
+  </si>
+  <si>
+    <t>First, the 4th Basic Plan for Wetland Conservation (2023–2027) proposes a coastal wetland restoration target of 7 km2 by 2027 and specifies a plan to expand the tidal flat vegetation restoration project to a scale of 60 km2 by 2027.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Second, the national goal presented in the "Toward Green Shipping by 2050" report submitted by the Korean government to the IMO states that the Blue Carbon sector aims to achieve a total CO2 absorption of 1,362 MtCO2eq by 2050 by restoring a total of 30km2 of tidal flats, utilizing abandoned salt and fish farms by 2050.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Accordingly, this study set the mid-to-long-term restoration pathway as follows: Restoring the Basic Plan's target of 7km2 between 2023 and 2037, and subsequently carrying out additional restoration until the cumulative restored area reaches 30km2 by 2050.</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -425,7 +594,7 @@
     <numFmt numFmtId="179" formatCode="_-* #,##0.0000_-;\-* #,##0.0000_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="180" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -543,6 +712,20 @@
     <font>
       <sz val="9"/>
       <color rgb="FF444444"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -726,15 +909,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -745,9 +921,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="177" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -755,31 +928,27 @@
     <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="178" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="180" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="179" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -802,23 +971,22 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="13" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="13" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="41" fontId="13" fillId="0" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="13" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="41" fontId="13" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="13" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="41" fontId="13" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -829,7 +997,7 @@
     <xf numFmtId="3" fontId="13" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="13" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="13" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -838,23 +1006,36 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="13" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="3" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="13" fillId="0" borderId="3" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="쉼표 [0]" xfId="2" builtinId="6"/>
@@ -876,9 +1057,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -916,9 +1097,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -951,26 +1132,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1003,26 +1167,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1196,9 +1343,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B65"/>
+  <dimension ref="A1:B77"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="15.25" customWidth="1"/>
     <col min="2" max="2" width="57.625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1211,42 +1359,42 @@
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B4" s="47" t="s">
+      <c r="B4" s="41" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B5" s="48">
+      <c r="B5" s="42">
         <v>2024</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B6" s="48" t="s">
+      <c r="B6" s="42" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B7" s="46" t="s">
+      <c r="B7" s="40" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B8" s="45" t="s">
-        <v>99</v>
+      <c r="B8" s="39" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="4" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1256,27 +1404,27 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B13" s="47" t="s">
+      <c r="B13" s="41" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B14" s="48">
+      <c r="B14" s="42">
         <v>2024</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="42" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B16" s="46" t="s">
+      <c r="B16" s="40" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B17" s="48" t="s">
+      <c r="B17" s="42" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1286,33 +1434,33 @@
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B20" s="47" t="s">
+      <c r="B20" s="41" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B21" s="48">
+      <c r="B21" s="42">
         <v>2024</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B22" s="48" t="s">
+      <c r="B22" s="42" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B23" s="46" t="s">
+      <c r="B23" s="40" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B24" s="45" t="s">
+      <c r="B24" s="39" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10" t="s">
+      <c r="A26" s="7"/>
+      <c r="B26" s="7" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1332,7 +1480,7 @@
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B30" s="30" t="s">
+      <c r="B30" s="26" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1341,161 +1489,218 @@
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B33" s="10" t="s">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B33" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B34" s="47" t="s">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B34" s="41" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B35" s="48">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B35" s="42">
         <v>2024</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B36" s="48" t="s">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B36" s="42" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B37" s="46" t="s">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B37" s="40" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B38" s="47" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B40" s="10" t="s">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B38" s="41" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B40" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B41" s="54" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B42" s="48">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B41" s="48" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B42" s="42">
         <v>2022</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B43" s="55" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B44" s="47" t="s">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B43" s="26" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B44" s="41" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" s="10" t="s">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B45" s="41"/>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B46" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B47" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B48" s="42">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B49" s="67" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B50" s="42"/>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="11" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="8" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="10" t="s">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="7" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="10" t="s">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A57" s="10" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A62" s="10" t="s">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A68" s="7" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A65" s="10"/>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A71" s="7" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A73" s="70" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" s="71" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="70" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" s="71" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="70" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" s="71" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="70" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" s="71" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="70"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B30" r:id="rId1" xr:uid="{E3C92502-A1D2-45B8-85DE-CCE90EDEF2CE}"/>
+    <hyperlink ref="B43" r:id="rId2" xr:uid="{8B0C0082-1835-4C72-9132-A2097D5281D8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -1508,258 +1713,258 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D2" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="11"/>
+      <c r="E2" s="8"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="14">
+      <c r="B3" s="10">
         <v>2015</v>
       </c>
-      <c r="C3" s="14">
+      <c r="C3" s="10">
         <v>2016</v>
       </c>
-      <c r="D3" s="14">
+      <c r="D3" s="10">
         <v>2017</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" s="10">
         <v>2018</v>
       </c>
-      <c r="F3" s="14">
+      <c r="F3" s="10">
         <v>2019</v>
       </c>
-      <c r="G3" s="49">
+      <c r="G3" s="43">
         <v>2020</v>
       </c>
-      <c r="H3" s="49">
+      <c r="H3" s="43">
         <v>2021</v>
       </c>
-      <c r="I3" s="49">
+      <c r="I3" s="43">
         <v>2022</v>
       </c>
-      <c r="J3" s="49">
+      <c r="J3" s="43">
         <v>2023</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="11">
         <v>23.178000000000001</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="11">
         <v>23.917000000000002</v>
       </c>
-      <c r="D4" s="15">
+      <c r="D4" s="11">
         <v>23.673999999999999</v>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="11">
         <v>23.088999999999999</v>
       </c>
-      <c r="F4" s="15">
+      <c r="F4" s="11">
         <v>23.413</v>
       </c>
-      <c r="G4" s="50">
+      <c r="G4" s="44">
         <v>23.17</v>
       </c>
-      <c r="H4" s="50">
+      <c r="H4" s="44">
         <v>20.6</v>
       </c>
-      <c r="I4" s="50">
+      <c r="I4" s="44">
         <v>19.170000000000002</v>
       </c>
-      <c r="J4" s="50">
+      <c r="J4" s="44">
         <v>21.11</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
+      <c r="A5" s="7"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="12" t="s">
+      <c r="B6" s="8"/>
+      <c r="C6" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D6" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="13">
         <f>AVERAGE($B$4:$F$4)</f>
         <v>23.4542</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="12" t="s">
+      <c r="B9" s="8"/>
+      <c r="C9" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D9" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="11">
+      <c r="A10" s="8">
         <v>2020</v>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="14">
         <v>10041.280000000001</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="12" t="s">
+      <c r="B12" s="8"/>
+      <c r="C12" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D12" t="s">
         <v>45</v>
       </c>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="11">
+      <c r="A13" s="8">
         <v>2020</v>
       </c>
-      <c r="B13" s="20">
+      <c r="B13" s="16">
         <v>6363.549</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="27">
+      <c r="A16" s="23">
         <f>($B7)/$B10</f>
         <v>2.3357779087925046E-3</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11" t="s">
+      <c r="B16" s="8"/>
+      <c r="C16" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="21">
+      <c r="A17" s="17">
         <f>$A16*$B10</f>
         <v>23.454200000000004</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="12" t="s">
+      <c r="B17" s="8"/>
+      <c r="C17" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D17" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="11"/>
+      <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="22">
+      <c r="A18" s="18">
         <f>$A17*10^3</f>
         <v>23454.200000000004</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D18" t="s">
@@ -1767,11 +1972,11 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="38">
+      <c r="A19" s="32">
         <f>$A18*$B$23</f>
         <v>57956.594726800016</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D19" t="s">
@@ -1779,7 +1984,7 @@
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="7" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1795,7 +2000,7 @@
       <c r="A23">
         <v>1</v>
       </c>
-      <c r="B23" s="23">
+      <c r="B23" s="19">
         <v>2.4710540000000001</v>
       </c>
     </row>
@@ -1821,10 +2026,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D2" t="s">
@@ -1832,69 +2037,69 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="14">
+      <c r="B3" s="10">
         <v>2015</v>
       </c>
-      <c r="C3" s="14">
+      <c r="C3" s="10">
         <v>2016</v>
       </c>
-      <c r="D3" s="14">
+      <c r="D3" s="10">
         <v>2017</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" s="10">
         <v>2018</v>
       </c>
-      <c r="F3" s="14">
+      <c r="F3" s="10">
         <v>2019</v>
       </c>
-      <c r="G3" s="49">
+      <c r="G3" s="43">
         <v>2020</v>
       </c>
-      <c r="H3" s="49">
+      <c r="H3" s="43">
         <v>2021</v>
       </c>
-      <c r="I3" s="49">
+      <c r="I3" s="43">
         <v>2022</v>
       </c>
-      <c r="J3" s="69"/>
+      <c r="J3" s="60"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="24">
+      <c r="B4" s="20">
         <v>166871</v>
       </c>
-      <c r="C4" s="24">
+      <c r="C4" s="20">
         <v>265684</v>
       </c>
-      <c r="D4" s="24">
+      <c r="D4" s="20">
         <v>183362</v>
       </c>
-      <c r="E4" s="24">
+      <c r="E4" s="20">
         <v>116931</v>
       </c>
-      <c r="F4" s="24">
+      <c r="F4" s="20">
         <v>100588</v>
       </c>
-      <c r="G4" s="51">
+      <c r="G4" s="45">
         <v>127700</v>
       </c>
-      <c r="H4" s="51">
+      <c r="H4" s="45">
         <v>106031</v>
       </c>
-      <c r="I4" s="51">
+      <c r="I4" s="45">
         <v>115528</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D6" t="s">
@@ -1905,30 +2110,30 @@
       <c r="A7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="21">
         <f>AVERAGE($B$4:$F$4)</f>
         <v>166687.20000000001</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C9" s="12"/>
+      <c r="C9" s="9"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B10" s="31">
+      <c r="B10" s="27">
         <f>$B$7/('Aff Ref'!B13*1000)</f>
         <v>2.6194062464200404E-2</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="7" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="38">
+      <c r="A13" s="32">
         <v>0</v>
       </c>
       <c r="B13" t="s">
@@ -1939,7 +2144,7 @@
       <c r="A16" s="1"/>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A29" s="26"/>
+      <c r="A29" s="22"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
@@ -1958,12 +2163,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="9" t="s">
         <v>52</v>
       </c>
       <c r="F2" t="s">
@@ -1971,42 +2176,42 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="14">
+      <c r="B3" s="10">
         <v>2016</v>
       </c>
-      <c r="C3" s="14">
+      <c r="C3" s="10">
         <v>2017</v>
       </c>
-      <c r="D3" s="14">
+      <c r="D3" s="10">
         <v>2018</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" s="10">
         <v>2019</v>
       </c>
-      <c r="F3" s="14">
+      <c r="F3" s="10">
         <v>2020</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="24">
+      <c r="B4" s="20">
         <v>1134</v>
       </c>
-      <c r="C4" s="24">
+      <c r="C4" s="20">
         <v>1632</v>
       </c>
-      <c r="D4" s="24">
+      <c r="D4" s="20">
         <v>1463</v>
       </c>
-      <c r="E4" s="24">
+      <c r="E4" s="20">
         <v>895</v>
       </c>
-      <c r="F4" s="24">
+      <c r="F4" s="20">
         <v>704</v>
       </c>
     </row>
@@ -2016,7 +2221,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="39">
+      <c r="A7" s="33">
         <f>AVERAGE($E$4:$F$4)/('Aff Ref'!B13*1000)</f>
         <v>1.2563743910827118E-4</v>
       </c>
@@ -2028,7 +2233,7 @@
       <c r="A8" s="1"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="7" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2050,13 +2255,13 @@
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.625" customWidth="1"/>
@@ -2073,58 +2278,55 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="7" t="s">
         <v>55</v>
       </c>
       <c r="B2"/>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D2" t="s">
         <v>36</v>
       </c>
-      <c r="E2" s="12"/>
+      <c r="E2" s="9"/>
       <c r="F2"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="10" t="s">
         <v>40</v>
       </c>
       <c r="F3"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="29">
+      <c r="B4" s="25">
         <v>163.30000000000001</v>
       </c>
-      <c r="C4" s="29">
+      <c r="C4" s="25">
         <v>155.9</v>
       </c>
-      <c r="D4" s="29">
+      <c r="D4" s="25">
         <v>138.30000000000001</v>
       </c>
       <c r="F4"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-    </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="7" t="s">
         <v>44</v>
       </c>
       <c r="B6"/>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D6" t="s">
@@ -2133,226 +2335,222 @@
       <c r="F6"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="10" t="s">
         <v>41</v>
       </c>
       <c r="F7"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="52">
+      <c r="B8" s="46">
         <v>1652736</v>
       </c>
-      <c r="C8" s="52">
+      <c r="C8" s="46">
         <v>483202</v>
       </c>
-      <c r="D8" s="53">
+      <c r="D8" s="47">
         <v>4162196</v>
       </c>
-      <c r="E8" s="52">
+      <c r="E8" s="46">
         <f>SUM($B$8:$D$8)</f>
         <v>6298134</v>
       </c>
-      <c r="F8" s="51" t="s">
+      <c r="F8" s="45" t="s">
         <v>95</v>
       </c>
-      <c r="G8" s="54"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
+      <c r="G8" s="48"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D10" t="s">
         <v>45</v>
       </c>
-      <c r="H10" s="12"/>
+      <c r="H10" s="9"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="40" t="s">
+      <c r="A11" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="41">
+      <c r="B11" s="35">
         <v>2011</v>
       </c>
-      <c r="C11" s="41">
+      <c r="C11" s="35">
         <v>2012</v>
       </c>
-      <c r="D11" s="41">
+      <c r="D11" s="35">
         <v>2013</v>
       </c>
-      <c r="E11" s="41">
+      <c r="E11" s="35">
         <v>2014</v>
       </c>
-      <c r="F11" s="41">
+      <c r="F11" s="35">
         <v>2015</v>
       </c>
-      <c r="G11" s="41">
+      <c r="G11" s="35">
         <v>2016</v>
       </c>
-      <c r="H11" s="57">
+      <c r="H11" s="50">
         <v>2017</v>
       </c>
-      <c r="I11" s="57">
+      <c r="I11" s="50">
         <v>2018</v>
       </c>
-      <c r="J11" s="57">
+      <c r="J11" s="50">
         <v>2019</v>
       </c>
-      <c r="K11" s="56">
+      <c r="K11" s="49">
         <v>2020</v>
       </c>
-      <c r="L11" s="56">
+      <c r="L11" s="49">
         <v>2021</v>
       </c>
-      <c r="M11" s="56">
+      <c r="M11" s="49">
         <v>2022</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="42">
+      <c r="B12" s="36">
         <v>459.964</v>
       </c>
-      <c r="C12" s="42">
+      <c r="C12" s="36">
         <v>415.21499999999997</v>
       </c>
-      <c r="D12" s="42">
+      <c r="D12" s="36">
         <v>370.61700000000002</v>
       </c>
-      <c r="E12" s="42">
+      <c r="E12" s="36">
         <v>293.33699999999999</v>
       </c>
-      <c r="F12" s="42">
+      <c r="F12" s="36">
         <v>279.15699999999998</v>
       </c>
-      <c r="G12" s="58">
+      <c r="G12" s="51">
         <v>283.59199999999998</v>
       </c>
-      <c r="H12" s="59">
+      <c r="H12" s="52">
         <v>306.49900000000002</v>
       </c>
-      <c r="I12" s="59">
+      <c r="I12" s="52">
         <v>255.02500000000001</v>
       </c>
-      <c r="J12" s="63">
+      <c r="J12" s="56">
         <v>210.62100000000001</v>
       </c>
-      <c r="K12" s="60">
+      <c r="K12" s="53">
         <v>228.78</v>
       </c>
-      <c r="L12" s="60">
+      <c r="L12" s="53">
         <v>209.16</v>
       </c>
-      <c r="M12" s="60">
+      <c r="M12" s="53">
         <v>224.53899999999999</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="40" t="s">
+      <c r="A13" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="B13" s="42">
+      <c r="B13" s="36">
         <v>71.022000000000006</v>
       </c>
-      <c r="C13" s="42">
+      <c r="C13" s="36">
         <v>65.173000000000002</v>
       </c>
-      <c r="D13" s="42">
+      <c r="D13" s="36">
         <v>69.256</v>
       </c>
-      <c r="E13" s="42">
+      <c r="E13" s="36">
         <v>54.654000000000003</v>
       </c>
-      <c r="F13" s="42">
+      <c r="F13" s="36">
         <v>50.322000000000003</v>
       </c>
-      <c r="G13" s="61">
+      <c r="G13" s="54">
         <v>51.484999999999999</v>
       </c>
-      <c r="H13" s="62">
+      <c r="H13" s="55">
         <v>52.985999999999997</v>
       </c>
-      <c r="I13" s="62">
+      <c r="I13" s="55">
         <v>41.805999999999997</v>
       </c>
-      <c r="J13" s="64">
+      <c r="J13" s="57">
         <v>44.359000000000002</v>
       </c>
-      <c r="K13" s="65">
+      <c r="K13" s="58">
         <v>37.811</v>
       </c>
-      <c r="L13" s="65">
+      <c r="L13" s="58">
         <v>35.911999999999999</v>
       </c>
-      <c r="M13" s="65">
+      <c r="M13" s="58">
         <v>33.878999999999998</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="40" t="s">
+      <c r="A14" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="42">
+      <c r="B14" s="36">
         <v>388.94200000000001</v>
       </c>
-      <c r="C14" s="42">
+      <c r="C14" s="36">
         <v>350.04199999999997</v>
       </c>
-      <c r="D14" s="42">
+      <c r="D14" s="36">
         <v>301.36099999999999</v>
       </c>
-      <c r="E14" s="42">
+      <c r="E14" s="36">
         <v>238.68299999999999</v>
       </c>
-      <c r="F14" s="42">
+      <c r="F14" s="36">
         <v>228.83500000000001</v>
       </c>
-      <c r="G14" s="61">
+      <c r="G14" s="54">
         <v>232.107</v>
       </c>
-      <c r="H14" s="61">
+      <c r="H14" s="54">
         <v>253.51300000000001</v>
       </c>
-      <c r="I14" s="61">
+      <c r="I14" s="54">
         <v>213.16499999999999</v>
       </c>
-      <c r="J14" s="58">
+      <c r="J14" s="51">
         <v>166.262</v>
       </c>
-      <c r="K14" s="65">
+      <c r="K14" s="58">
         <v>190.96899999999999</v>
       </c>
-      <c r="L14" s="65">
+      <c r="L14" s="58">
         <v>173.24799999999999</v>
       </c>
-      <c r="M14" s="65">
+      <c r="M14" s="58">
         <v>19.66</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
       <c r="C15" s="4"/>
       <c r="E15" s="4"/>
     </row>
@@ -2362,8 +2560,8 @@
       </c>
       <c r="C16" s="4"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="28">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A17" s="24">
         <f>$D$8/$E$8</f>
         <v>0.66086177270918656</v>
       </c>
@@ -2371,163 +2569,88 @@
         <v>47</v>
       </c>
       <c r="C17" s="4"/>
-      <c r="F17" s="66"/>
-      <c r="G17" s="67"/>
-      <c r="H17" s="67"/>
-      <c r="I17" s="67"/>
-      <c r="J17" s="67"/>
-      <c r="K17" s="67"/>
-      <c r="L17" s="67"/>
-      <c r="M17" s="67"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="43">
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A18" s="37">
         <f>AVERAGE(F14:J14)*1000/$D$8</f>
         <v>5.2562733710762304E-2</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="F18" s="66"/>
-      <c r="G18" s="67"/>
-      <c r="H18" s="67"/>
-      <c r="I18" s="67"/>
-      <c r="J18" s="67"/>
-      <c r="K18" s="67"/>
-      <c r="L18" s="67"/>
-      <c r="M18" s="67"/>
-      <c r="N18" s="67"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="36">
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A19">
         <f>A18*D8</f>
         <v>218776.40000000002</v>
       </c>
       <c r="B19" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="F19" s="66"/>
-      <c r="G19" s="68"/>
-      <c r="H19" s="68"/>
-      <c r="I19" s="68"/>
-      <c r="J19" s="68"/>
-      <c r="K19" s="68"/>
-      <c r="L19" s="68"/>
-      <c r="M19" s="68"/>
-      <c r="N19" s="67"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="37">
+      <c r="G19" s="59"/>
+      <c r="H19" s="59"/>
+      <c r="I19" s="59"/>
+      <c r="J19" s="59"/>
+      <c r="K19" s="59"/>
+      <c r="L19" s="59"/>
+      <c r="M19" s="59"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A20" s="31">
         <f>A19*'Aff Ref'!B23</f>
         <v>540608.2983256001</v>
       </c>
       <c r="B20"/>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D20" t="s">
         <v>62</v>
       </c>
-      <c r="F20" s="66"/>
-      <c r="G20" s="68"/>
-      <c r="H20" s="68"/>
-      <c r="I20" s="68"/>
-      <c r="J20" s="68"/>
-      <c r="K20" s="68"/>
-      <c r="L20" s="68"/>
-      <c r="M20" s="68"/>
-      <c r="N20" s="67"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="F21" s="66"/>
-      <c r="G21" s="68"/>
-      <c r="H21" s="68"/>
-      <c r="I21" s="68"/>
-      <c r="J21" s="68"/>
-      <c r="K21" s="68"/>
-      <c r="L21" s="68"/>
-      <c r="M21" s="68"/>
-      <c r="N21" s="67"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="G20" s="59"/>
+      <c r="H20" s="59"/>
+      <c r="I20" s="59"/>
+      <c r="J20" s="59"/>
+      <c r="K20" s="59"/>
+      <c r="L20" s="59"/>
+      <c r="M20" s="59"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="G21" s="59"/>
+      <c r="H21" s="59"/>
+      <c r="I21" s="59"/>
+      <c r="J21" s="59"/>
+      <c r="K21" s="59"/>
+      <c r="L21" s="59"/>
+      <c r="M21" s="59"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="F22" s="66"/>
-      <c r="G22" s="67"/>
-      <c r="H22" s="67"/>
-      <c r="I22" s="67"/>
-      <c r="J22" s="67"/>
-      <c r="K22" s="67"/>
-      <c r="L22" s="67"/>
-      <c r="M22" s="67"/>
-      <c r="N22" s="67"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B23"/>
-      <c r="F23" s="66"/>
-      <c r="G23" s="67"/>
-      <c r="H23" s="67"/>
-      <c r="I23" s="67"/>
-      <c r="J23" s="67"/>
-      <c r="K23" s="67"/>
-      <c r="L23" s="67"/>
-      <c r="M23" s="67"/>
-      <c r="N23" s="67"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B24"/>
-      <c r="F24" s="66"/>
-      <c r="G24" s="67"/>
-      <c r="H24" s="67"/>
-      <c r="I24" s="67"/>
-      <c r="J24" s="67"/>
-      <c r="K24" s="67"/>
-      <c r="L24" s="67"/>
-      <c r="M24" s="67"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="6"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A25" s="5"/>
       <c r="B25"/>
-      <c r="F25" s="66"/>
-      <c r="G25" s="67"/>
-      <c r="H25" s="67"/>
-      <c r="I25" s="67"/>
-      <c r="J25" s="67"/>
-      <c r="K25" s="67"/>
-      <c r="L25" s="67"/>
-      <c r="M25" s="67"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="F26" s="66"/>
-      <c r="G26" s="67"/>
-      <c r="H26" s="67"/>
-      <c r="I26" s="67"/>
-      <c r="J26" s="67"/>
-      <c r="K26" s="67"/>
-      <c r="L26" s="67"/>
-      <c r="M26" s="67"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="F27" s="66"/>
-      <c r="G27" s="67"/>
-      <c r="H27" s="67"/>
-      <c r="I27" s="67"/>
-      <c r="J27" s="67"/>
-      <c r="K27" s="67"/>
-      <c r="L27" s="67"/>
-      <c r="M27" s="67"/>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="26"/>
+      <c r="A37" s="22"/>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" s="6"/>
+      <c r="A40" s="5"/>
       <c r="B40"/>
     </row>
   </sheetData>
@@ -2541,173 +2664,173 @@
   <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.125" style="11" customWidth="1"/>
-    <col min="2" max="6" width="9.125" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="11"/>
+    <col min="1" max="1" width="17.125" style="8" customWidth="1"/>
+    <col min="2" max="6" width="9.125" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="7" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="33">
+      <c r="B3" s="28">
         <v>2015</v>
       </c>
-      <c r="C3" s="33">
+      <c r="C3" s="28">
         <v>2016</v>
       </c>
-      <c r="D3" s="33">
+      <c r="D3" s="28">
         <v>2017</v>
       </c>
-      <c r="E3" s="33">
+      <c r="E3" s="28">
         <v>2018</v>
       </c>
-      <c r="F3" s="33">
+      <c r="F3" s="28">
         <v>2019</v>
       </c>
-      <c r="G3" s="70">
+      <c r="G3" s="61">
         <v>2020</v>
       </c>
-      <c r="H3" s="70">
+      <c r="H3" s="61">
         <v>2021</v>
       </c>
-      <c r="I3" s="70">
+      <c r="I3" s="61">
         <v>2022</v>
       </c>
-      <c r="J3" s="70">
+      <c r="J3" s="61">
         <v>2023</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="11">
         <v>51.4</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="11">
         <v>48.2</v>
       </c>
-      <c r="D4" s="15">
+      <c r="D4" s="11">
         <v>54.5</v>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="11">
         <v>46.3</v>
       </c>
-      <c r="F4" s="15">
+      <c r="F4" s="11">
         <v>27.4</v>
       </c>
-      <c r="G4" s="71">
+      <c r="G4" s="62">
         <v>58</v>
       </c>
-      <c r="H4" s="50">
+      <c r="H4" s="44">
         <v>86.5</v>
       </c>
-      <c r="I4" s="50">
+      <c r="I4" s="44">
         <v>164.1</v>
       </c>
-      <c r="J4" s="50">
+      <c r="J4" s="44">
         <v>319.2</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="C5" s="12"/>
+      <c r="A5" s="7"/>
+      <c r="C5" s="9"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="G6" s="34"/>
+      <c r="G6" s="29"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="14">
         <f>AVERAGE($B$4:$F$4)/10^3</f>
         <v>4.5559999999999996E-2</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="8" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="11">
+      <c r="A10" s="8">
         <v>2020</v>
       </c>
-      <c r="B10" s="20">
+      <c r="B10" s="16">
         <v>6363.549</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="7" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="21">
+      <c r="A13" s="17">
         <f>B7</f>
         <v>4.5559999999999996E-2</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="8" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="22">
+      <c r="A14" s="18">
         <f>$A13*10^3</f>
         <v>45.559999999999995</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="35">
+      <c r="A15" s="30">
         <f>$A14*'Aff Ref'!$B$23</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="8" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2718,6 +2841,171 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{166CF33E-7EFA-4C86-96D0-4CC055EC0D44}">
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="66" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="65" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="63" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" s="63" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6">
+        <f>7*B15</f>
+        <v>1729.7376669999999</v>
+      </c>
+      <c r="C6">
+        <f>30*B15</f>
+        <v>7413.1614300000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="33" x14ac:dyDescent="0.3">
+      <c r="A7" s="64" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="64" t="s">
+        <v>106</v>
+      </c>
+      <c r="B8">
+        <f>SUM(B6:B7)</f>
+        <v>1729.7376669999999</v>
+      </c>
+      <c r="C8">
+        <f>SUM(C6:C7)</f>
+        <v>7413.1614300000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="33" x14ac:dyDescent="0.3">
+      <c r="A10" s="64" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="64" t="s">
+        <v>120</v>
+      </c>
+      <c r="B11">
+        <f>B8/(2027-2023+1)</f>
+        <v>345.9475334</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="64" t="s">
+        <v>121</v>
+      </c>
+      <c r="B12">
+        <f>(C6-B6)/(2050-2028+1)</f>
+        <v>247.10538100000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>1</v>
+      </c>
+      <c r="B15">
+        <v>247.10538099999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>1</v>
+      </c>
+      <c r="B17">
+        <v>2.4710538099999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="68" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="69" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="69" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -3427,249 +3715,283 @@
         <v>0</v>
       </c>
       <c r="C6">
+        <f>B6</f>
         <v>0</v>
       </c>
       <c r="D6">
+        <f t="shared" ref="D6:AJ6" si="0">C6</f>
         <v>0</v>
       </c>
       <c r="E6">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F6">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G6">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H6">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <f>'Peatland Restoration'!B11</f>
+        <v>345.9475334</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>345.9475334</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>345.9475334</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>345.9475334</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>345.9475334</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <f>'Peatland Restoration'!B12</f>
+        <v>247.10538100000002</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="T6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="V6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="W6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="X6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="Y6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="Z6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="AA6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="AB6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="AC6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="AD6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="AE6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="AF6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="AG6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="AH6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="AI6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
       <c r="AJ6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>247.10538100000002</v>
       </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="44">
+      <c r="B7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="C7" s="44">
+      <c r="C7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="D7" s="44">
+      <c r="D7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="E7" s="44">
+      <c r="E7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="F7" s="44">
+      <c r="F7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="G7" s="44">
+      <c r="G7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="H7" s="44">
+      <c r="H7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="I7" s="44">
+      <c r="I7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="J7" s="44">
+      <c r="J7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="K7" s="44">
+      <c r="K7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="L7" s="44">
+      <c r="L7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="M7" s="44">
+      <c r="M7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="N7" s="44">
+      <c r="N7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="O7" s="44">
+      <c r="O7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="P7" s="44">
+      <c r="P7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="Q7" s="44">
+      <c r="Q7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="R7" s="44">
+      <c r="R7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="S7" s="44">
+      <c r="S7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="T7" s="44">
+      <c r="T7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="U7" s="44">
+      <c r="U7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="V7" s="44">
+      <c r="V7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="W7" s="44">
+      <c r="W7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="X7" s="44">
+      <c r="X7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="Y7" s="44">
+      <c r="Y7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="Z7" s="44">
+      <c r="Z7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="AA7" s="44">
+      <c r="AA7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="AB7" s="44">
+      <c r="AB7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="AC7" s="44">
+      <c r="AC7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="AD7" s="44">
+      <c r="AD7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="AE7" s="44">
+      <c r="AE7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="AF7" s="44">
+      <c r="AF7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="AG7" s="44">
+      <c r="AG7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="AH7" s="44">
+      <c r="AH7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="AI7" s="44">
+      <c r="AI7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
-      <c r="AJ7" s="44">
+      <c r="AJ7" s="38">
         <f>'Forest Restoration'!$A$15</f>
         <v>112.58122023999999</v>
       </c>
@@ -3681,6 +4003,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -3824,29 +4161,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C2455F5-A366-48C6-823F-E2E85D89160A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FADA85B9-6D15-46DA-8645-319EAC5A0213}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B851C5AF-E5C5-495B-9C6C-B733EF4C3B22}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B851C5AF-E5C5-495B-9C6C-B733EF4C3B22}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FADA85B9-6D15-46DA-8645-319EAC5A0213}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C2455F5-A366-48C6-823F-E2E85D89160A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>